<commit_message>
review of aa library
</commit_message>
<xml_diff>
--- a/pepfoundry/project/core/amino_acids_library.xlsx
+++ b/pepfoundry/project/core/amino_acids_library.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielgarzonotero/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC822AC-8FF1-F341-A42C-28B42092C152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D8F0CA-3856-3448-B576-D8A339DB6E2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1601,7 +1601,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1097" uniqueCount="616">
   <si>
     <t>#</t>
   </si>
@@ -12863,6 +12863,12 @@
       <c r="I120" s="2" t="e" vm="119">
         <v>#VALUE!</v>
       </c>
+      <c r="J120" s="21" t="s">
+        <v>398</v>
+      </c>
+      <c r="K120" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="121" spans="1:11" ht="95.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="2">

</xml_diff>